<commit_message>
Live Katalog-Korrektur via Streamlit Data Editor
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -815,7 +815,11 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>-</t>
@@ -932,7 +936,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -940,7 +944,11 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>-</t>
@@ -1057,7 +1065,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1333,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2228,7 +2236,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2615,7 +2623,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">

</xml_diff>